<commit_message>
Add request response evidence to bug register
</commit_message>
<xml_diff>
--- a/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
+++ b/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Bug Register'!A1:K13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Bug Register'!A1:L13</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L13"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -412,8 +412,9 @@
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" customWidth="1"/>
     <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="40.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -445,9 +446,12 @@
         <v>Evidence</v>
       </c>
       <c r="J1" t="str">
+        <v>Request/Response or Console Evidence</v>
+      </c>
+      <c r="K1" t="str">
         <v>Status</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Recommendation</v>
       </c>
     </row>
@@ -480,9 +484,12 @@
         <v>tests/pricing-consistency.spec.ts; reports/TASK-02-BUG-REPORT.md</v>
       </c>
       <c r="J2" t="str">
+        <v>Pricing extraction: monthlyPrice=12, annualPrice=144, statedSaving=20; calculatedSaving=0.</v>
+      </c>
+      <c r="K2" t="str">
         <v>Confirmed defect</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>Centralize pricing values and correct either the monthly base price or annual discount label.</v>
       </c>
     </row>
@@ -515,9 +522,12 @@
         <v>tests/pricing-consistency.spec.ts; tests/faq-pricing.spec.ts</v>
       </c>
       <c r="J3" t="str">
+        <v>Pricing page text contains $12/month; FAQ pricing answer contains $15.</v>
+      </c>
+      <c r="K3" t="str">
         <v>Confirmed inconsistency</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>Use one shared pricing source for Pricing, FAQ, checkout, and marketing content.</v>
       </c>
     </row>
@@ -550,9 +560,12 @@
         <v>tests/contact-inspection.spec.ts; tests/contact-input-security.spec.ts</v>
       </c>
       <c r="J4" t="str">
+        <v>Contact POST returned 200; fields reported maxLength=-1; no reflected script text observed.</v>
+      </c>
+      <c r="K4" t="str">
         <v>Observation; server limit not independently verified</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>Define and test explicit server-side and client-side field limits.</v>
       </c>
     </row>
@@ -585,9 +598,12 @@
         <v>tests/compatibility.spec.ts; reports/TASK-02-BUG-REPORT.md</v>
       </c>
       <c r="J5" t="str">
+        <v>Firefox navigation returned HTTP 200; page remained on loading spinner and body content was empty.</v>
+      </c>
+      <c r="K5" t="str">
         <v>Confirmed compatibility failure</v>
       </c>
-      <c r="K5" t="str">
+      <c r="L5" t="str">
         <v>Investigate Firefox-specific hydration, JavaScript, or resource-loading behavior.</v>
       </c>
     </row>
@@ -620,9 +636,12 @@
         <v>tests/contact-submission.spec.ts; TESTING-TODO.md</v>
       </c>
       <c r="J6" t="str">
+        <v>POST /api/communications/send returned 200; Gmail marker search found no matching message.</v>
+      </c>
+      <c r="K6" t="str">
         <v>Blocked: recipient mailbox unavailable</v>
       </c>
-      <c r="K6" t="str">
+      <c r="L6" t="str">
         <v>Identify or configure a controlled recipient mailbox and repeat marker-based delivery verification.</v>
       </c>
     </row>
@@ -655,9 +674,12 @@
         <v>reports/lighthouse-api.json; README.md</v>
       </c>
       <c r="J7" t="str">
+        <v>Lighthouse document request for /api returned 401 ERRORED_DOCUMENT_REQUEST.</v>
+      </c>
+      <c r="K7" t="str">
         <v>Blocked by protected route</v>
       </c>
-      <c r="K7" t="str">
+      <c r="L7" t="str">
         <v>Keep the 401 as evidence or audit /api-platform separately for public documentation performance.</v>
       </c>
     </row>
@@ -690,9 +712,12 @@
         <v>reports/lighthouse-home.json; reports/TASK-02-BUG-REPORT.md</v>
       </c>
       <c r="J8" t="str">
+        <v>Lighthouse captured FCP/LCP/CLS/TBT/Speed Index/root response time; INP/FID was unavailable.</v>
+      </c>
+      <c r="K8" t="str">
         <v>Deferred: metric unavailable</v>
       </c>
-      <c r="K8" t="str">
+      <c r="L8" t="str">
         <v>Use field/RUM data if INP is required; do not infer INP/FID from other metrics.</v>
       </c>
     </row>
@@ -725,9 +750,12 @@
         <v>tests/task01/free-tier-quota.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
       <c r="J9" t="str">
+        <v>Free account UI displayed: Out of messages; 5 messages every 5 hours; reset countdown approximately 5 hours.</v>
+      </c>
+      <c r="K9" t="str">
         <v>Partial; state-dependent verification deferred</v>
       </c>
-      <c r="K9" t="str">
+      <c r="L9" t="str">
         <v>Repeat with a genuinely fresh quota bucket and reconcile the product window with the assignment wording.</v>
       </c>
     </row>
@@ -760,9 +788,12 @@
         <v>tests/task01/upload-integrity.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
       <c r="J10" t="str">
+        <v>Upload UI rendered PDF/CSV/SVG attachment chips; parsing request was not completed due to state-dependent limit.</v>
+      </c>
+      <c r="K10" t="str">
         <v>Partial; processing verification deferred</v>
       </c>
-      <c r="K10" t="str">
+      <c r="L10" t="str">
         <v>Repeat with available message quota and controlled fixtures, then validate extracted values and errors.</v>
       </c>
     </row>
@@ -795,9 +826,12 @@
         <v>tests/task01/memory-incognito.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
       <c r="J11" t="str">
+        <v>Memory panel opened; empty state observed; Incognito control visible and activatable.</v>
+      </c>
+      <c r="K11" t="str">
         <v>Partial; state-dependent verification deferred</v>
       </c>
-      <c r="K11" t="str">
+      <c r="L11" t="str">
         <v>Repeat with a fresh usable conversation state; document server-backup deletion as client-side unverifiable.</v>
       </c>
     </row>
@@ -830,9 +864,12 @@
         <v>tests/task01/developer-api-authenticated.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
       <c r="J12" t="str">
+        <v>POST /v1/chat/completions with accepted API key returned 402 Insufficient balance; invalid model returned 400.</v>
+      </c>
+      <c r="K12" t="str">
         <v>Partial; zero-balance verification boundary</v>
       </c>
-      <c r="K12" t="str">
+      <c r="L12" t="str">
         <v>Repeat with an approved funded test key and minimal token budget.</v>
       </c>
     </row>
@@ -865,16 +902,19 @@
         <v>tests/task01/negative-boundary.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
       <c r="J13" t="str">
+        <v>Authenticated UI probe exposed account menu but no editable Settings/Account/Billing form controls.</v>
+      </c>
+      <c r="K13" t="str">
         <v>Deferred: surface not exposed</v>
       </c>
-      <c r="K13" t="str">
+      <c r="L13" t="str">
         <v>Locate the product routes or enable the relevant surface, then add field-level boundary tests.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K13"/>
+  <autoFilter ref="A1:L13"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Organize Task 02 into dedicated folders
</commit_message>
<xml_diff>
--- a/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
+++ b/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
@@ -481,7 +481,7 @@
         <v>$12 x 12 = $144, so the displayed annual price represents 0% saving, not 20%.</v>
       </c>
       <c r="I2" t="str">
-        <v>tests/pricing-consistency.spec.ts; reports/TASK-02-BUG-REPORT.md</v>
+        <v>tests/task02/pricing-consistency.spec.ts; reports/task02/TASK-02-BUG-REPORT.md</v>
       </c>
       <c r="J2" t="str">
         <v>Pricing extraction: monthlyPrice=12, annualPrice=144, statedSaving=20; calculatedSaving=0.</v>
@@ -519,7 +519,7 @@
         <v>Pricing shows $12/month while FAQ references $15/month.</v>
       </c>
       <c r="I3" t="str">
-        <v>tests/pricing-consistency.spec.ts; tests/faq-pricing.spec.ts</v>
+        <v>tests/task02/pricing-consistency.spec.ts; tests/task02/faq-pricing.spec.ts</v>
       </c>
       <c r="J3" t="str">
         <v>Pricing page text contains $12/month; FAQ pricing answer contains $15.</v>
@@ -557,7 +557,7 @@
         <v>Fields exposed no client-side maxlength; unusual input returned without server error or reflected script.</v>
       </c>
       <c r="I4" t="str">
-        <v>tests/contact-inspection.spec.ts; tests/contact-input-security.spec.ts</v>
+        <v>tests/task02/contact-inspection.spec.ts; tests/task02/contact-input-security.spec.ts</v>
       </c>
       <c r="J4" t="str">
         <v>Contact POST returned 200; fields reported maxLength=-1; no reflected script text observed.</v>
@@ -595,7 +595,7 @@
         <v>Firefox returned 200 but remained on the loading spinner with no rendered body content.</v>
       </c>
       <c r="I5" t="str">
-        <v>tests/compatibility.spec.ts; reports/TASK-02-BUG-REPORT.md</v>
+        <v>tests/task02/compatibility.spec.ts; reports/task02/TASK-02-BUG-REPORT.md</v>
       </c>
       <c r="J5" t="str">
         <v>Firefox navigation returned HTTP 200; page remained on loading spinner and body content was empty.</v>
@@ -633,7 +633,7 @@
         <v>API/UI submission returned success, but recipient delivery could not be independently verified.</v>
       </c>
       <c r="I6" t="str">
-        <v>tests/contact-submission.spec.ts; TESTING-TODO.md</v>
+        <v>tests/task02/contact-submission.spec.ts; TESTING-TODO.md</v>
       </c>
       <c r="J6" t="str">
         <v>POST /api/communications/send returned 200; Gmail marker search found no matching message.</v>
@@ -671,7 +671,7 @@
         <v>The route returned 401, so performance metrics were unavailable; /api-platform is the public documentation page.</v>
       </c>
       <c r="I7" t="str">
-        <v>reports/lighthouse-api.json; README.md</v>
+        <v>reports/task02/lighthouse-api.json; README.md</v>
       </c>
       <c r="J7" t="str">
         <v>Lighthouse document request for /api returned 401 ERRORED_DOCUMENT_REQUEST.</v>
@@ -709,7 +709,7 @@
         <v>FCP, LCP, CLS, TBT, Speed Index, and root response time were available; INP/FID was unavailable in lab evidence.</v>
       </c>
       <c r="I8" t="str">
-        <v>reports/lighthouse-home.json; reports/TASK-02-BUG-REPORT.md</v>
+        <v>reports/task02/lighthouse-home.json; reports/task02/TASK-02-BUG-REPORT.md</v>
       </c>
       <c r="J8" t="str">
         <v>Lighthouse captured FCP/LCP/CLS/TBT/Speed Index/root response time; INP/FID was unavailable.</v>

</xml_diff>

<commit_message>
Confirm contact-form delivery via reply evidence; add SLA timing finding
</commit_message>
<xml_diff>
--- a/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
+++ b/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Bug Register'!A1:L13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Bug Register'!A1:L14</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -615,7 +615,7 @@
         <v>Task 02</v>
       </c>
       <c r="C6" t="str">
-        <v>Medium</v>
+        <v>Informational</v>
       </c>
       <c r="D6" t="str">
         <v>Contact delivery</v>
@@ -624,68 +624,68 @@
         <v>https://backend.thaura.ai/api/communications/send</v>
       </c>
       <c r="F6" t="str">
-        <v>Submit a uniquely marked valid Contact form message and search the controlled inbox.</v>
+        <v>Submit a valid Contact form message and check for delivery confirmation via reply.</v>
       </c>
       <c r="G6" t="str">
         <v>Submitted data is received by the configured recipient.</v>
       </c>
       <c r="H6" t="str">
-        <v>API/UI submission returned success, but recipient delivery could not be independently verified.</v>
+        <v>API/UI submission returned success; a manual submission received a reply from info@thaura.ai quoting the exact submitted Name, Email, Subject, and Message, confirming end-to-end delivery.</v>
       </c>
       <c r="I6" t="str">
-        <v>tests/task02/contact-submission.spec.ts; TESTING-TODO.md</v>
+        <v>tests/task02/contact-submission.spec.ts; TESTING-TODO.md; reply email from info@thaura.ai dated 2026-09-16</v>
       </c>
       <c r="J6" t="str">
-        <v>POST /api/communications/send returned 200; Gmail marker search found no matching message.</v>
+        <v>POST /api/communications/send returned 200; reply from info@thaura.ai quoted the exact submitted Name/Email/Subject/Message, confirming delivery.</v>
       </c>
       <c r="K6" t="str">
-        <v>Blocked: recipient mailbox unavailable</v>
+        <v>Confirmed: delivery verified</v>
       </c>
       <c r="L6" t="str">
-        <v>Identify or configure a controlled recipient mailbox and repeat marker-based delivery verification.</v>
+        <v>No further action; delivery is confirmed. Consider a controlled mailbox for repeatable automated verification.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>T02-F-006</v>
+        <v>T02-F-008</v>
       </c>
       <c r="B7" t="str">
         <v>Task 02</v>
       </c>
       <c r="C7" t="str">
-        <v>Informational</v>
+        <v>Low</v>
       </c>
       <c r="D7" t="str">
-        <v>Lighthouse API audit</v>
+        <v>Contact response SLA</v>
       </c>
       <c r="E7" t="str">
-        <v>https://thaura.ai/api</v>
+        <v>https://thaura.ai/contact</v>
       </c>
       <c r="F7" t="str">
-        <v>Run the configured Lighthouse API audit anonymously.</v>
+        <v>Submit a valid Contact form message, note the timestamp, and measure time until a reply arrives.</v>
       </c>
       <c r="G7" t="str">
-        <v>Key-page Lighthouse metrics are captured.</v>
+        <v>A reply arrives within the page's stated 24-hour commitment.</v>
       </c>
       <c r="H7" t="str">
-        <v>The route returned 401, so performance metrics were unavailable; /api-platform is the public documentation page.</v>
+        <v>A reply arrived approximately 44 hours after submission, exceeding the stated 24-hour commitment.</v>
       </c>
       <c r="I7" t="str">
-        <v>reports/task02/lighthouse-api.json; README.md</v>
+        <v>Reply email from info@thaura.ai dated 2026-09-16 14:31 responding to a submission dated 2026-09-14 18:15:55</v>
       </c>
       <c r="J7" t="str">
-        <v>Lighthouse document request for /api returned 401 ERRORED_DOCUMENT_REQUEST.</v>
+        <v>Submission at 2026-09-14 18:15:55 received a reply at 2026-09-16 14:31, approximately 44 hours later, versus the page's stated 24-hour commitment.</v>
       </c>
       <c r="K7" t="str">
-        <v>Blocked by protected route</v>
+        <v>Observation: single instance, not a confirmed pattern</v>
       </c>
       <c r="L7" t="str">
-        <v>Keep the 401 as evidence or audit /api-platform separately for public documentation performance.</v>
+        <v>Resource the Contact inbox to meet the stated SLA, or update the displayed SLA text to match actual response times.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>T02-F-007</v>
+        <v>T02-F-006</v>
       </c>
       <c r="B8" t="str">
         <v>Task 02</v>
@@ -694,74 +694,74 @@
         <v>Informational</v>
       </c>
       <c r="D8" t="str">
-        <v>Performance metrics</v>
+        <v>Lighthouse API audit</v>
       </c>
       <c r="E8" t="str">
-        <v>https://thaura.ai/</v>
+        <v>https://thaura.ai/api</v>
       </c>
       <c r="F8" t="str">
-        <v>Review stored Lighthouse lab metrics.</v>
+        <v>Run the configured Lighthouse API audit anonymously.</v>
       </c>
       <c r="G8" t="str">
-        <v>Requested Core Web Vitals are reported where supported.</v>
+        <v>Key-page Lighthouse metrics are captured.</v>
       </c>
       <c r="H8" t="str">
-        <v>FCP, LCP, CLS, TBT, Speed Index, and root response time were available; INP/FID was unavailable in lab evidence.</v>
+        <v>The route returned 401, so performance metrics were unavailable; /api-platform is the public documentation page.</v>
       </c>
       <c r="I8" t="str">
-        <v>reports/task02/lighthouse-home.json; reports/task02/TASK-02-BUG-REPORT.md</v>
+        <v>reports/task02/lighthouse-api.json; README.md</v>
       </c>
       <c r="J8" t="str">
-        <v>Lighthouse captured FCP/LCP/CLS/TBT/Speed Index/root response time; INP/FID was unavailable.</v>
+        <v>Lighthouse document request for /api returned 401 ERRORED_DOCUMENT_REQUEST.</v>
       </c>
       <c r="K8" t="str">
-        <v>Deferred: metric unavailable</v>
+        <v>Blocked by protected route</v>
       </c>
       <c r="L8" t="str">
-        <v>Use field/RUM data if INP is required; do not infer INP/FID from other metrics.</v>
+        <v>Keep the 401 as evidence or audit /api-platform separately for public documentation performance.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>T01-F-001</v>
+        <v>T02-F-007</v>
       </c>
       <c r="B9" t="str">
-        <v>Task 01</v>
+        <v>Task 02</v>
       </c>
       <c r="C9" t="str">
-        <v>Medium</v>
+        <v>Informational</v>
       </c>
       <c r="D9" t="str">
-        <v>Free-tier quota window</v>
+        <v>Performance metrics</v>
       </c>
       <c r="E9" t="str">
         <v>https://thaura.ai/</v>
       </c>
       <c r="F9" t="str">
-        <v>Open a Free account after quota exhaustion and inspect the limit message.</v>
+        <v>Review stored Lighthouse lab metrics.</v>
       </c>
       <c r="G9" t="str">
-        <v>The documented 5-message/2-hour behavior is confirmed.</v>
+        <v>Requested Core Web Vitals are reported where supported.</v>
       </c>
       <c r="H9" t="str">
-        <v>The product displayed 5 messages every 5 hours; a fresh #5/#6 boundary run was unavailable.</v>
+        <v>FCP, LCP, CLS, TBT, Speed Index, and root response time were available; INP/FID was unavailable in lab evidence.</v>
       </c>
       <c r="I9" t="str">
-        <v>tests/task01/free-tier-quota.spec.ts; reports/task01/TASK-01-REPORT.md</v>
+        <v>reports/task02/lighthouse-home.json; reports/task02/TASK-02-BUG-REPORT.md</v>
       </c>
       <c r="J9" t="str">
-        <v>Free account UI displayed: Out of messages; 5 messages every 5 hours; reset countdown approximately 5 hours.</v>
+        <v>Lighthouse captured FCP/LCP/CLS/TBT/Speed Index/root response time; INP/FID was unavailable.</v>
       </c>
       <c r="K9" t="str">
-        <v>Partial; state-dependent verification deferred</v>
+        <v>Deferred: metric unavailable</v>
       </c>
       <c r="L9" t="str">
-        <v>Repeat with a genuinely fresh quota bucket and reconcile the product window with the assignment wording.</v>
+        <v>Use field/RUM data if INP is required; do not infer INP/FID from other metrics.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>T01-F-002</v>
+        <v>T01-F-001</v>
       </c>
       <c r="B10" t="str">
         <v>Task 01</v>
@@ -770,36 +770,36 @@
         <v>Medium</v>
       </c>
       <c r="D10" t="str">
-        <v>Upload data integrity</v>
+        <v>Free-tier quota window</v>
       </c>
       <c r="E10" t="str">
         <v>https://thaura.ai/</v>
       </c>
       <c r="F10" t="str">
-        <v>Select PDF, CSV, image, corrupted, empty, oversized, and password-protected fixtures; request analysis.</v>
+        <v>Open a Free account after quota exhaustion and inspect the limit message.</v>
       </c>
       <c r="G10" t="str">
-        <v>Parsed content is accurate and invalid files return clear errors without silent failure.</v>
+        <v>The documented 5-message/2-hour behavior is confirmed.</v>
       </c>
       <c r="H10" t="str">
-        <v>Upload control accepted safe fixtures, but assistant-side parsing and full invalid-file processing were not completed.</v>
+        <v>The product displayed 5 messages every 5 hours; a fresh #5/#6 boundary run was unavailable.</v>
       </c>
       <c r="I10" t="str">
-        <v>tests/task01/upload-integrity.spec.ts; reports/task01/TASK-01-REPORT.md</v>
+        <v>tests/task01/free-tier-quota.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
       <c r="J10" t="str">
-        <v>Upload UI rendered PDF/CSV/SVG attachment chips; parsing request was not completed due to state-dependent limit.</v>
+        <v>Free account UI displayed: Out of messages; 5 messages every 5 hours; reset countdown approximately 5 hours.</v>
       </c>
       <c r="K10" t="str">
-        <v>Partial; processing verification deferred</v>
+        <v>Partial; state-dependent verification deferred</v>
       </c>
       <c r="L10" t="str">
-        <v>Repeat with available message quota and controlled fixtures, then validate extracted values and errors.</v>
+        <v>Repeat with a genuinely fresh quota bucket and reconcile the product window with the assignment wording.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>T01-F-003</v>
+        <v>T01-F-002</v>
       </c>
       <c r="B11" t="str">
         <v>Task 01</v>
@@ -808,36 +808,36 @@
         <v>Medium</v>
       </c>
       <c r="D11" t="str">
-        <v>Memory and Incognito</v>
+        <v>Upload data integrity</v>
       </c>
       <c r="E11" t="str">
         <v>https://thaura.ai/</v>
       </c>
       <c r="F11" t="str">
-        <v>Store a fact in normal mode, retrieve it in a new chat, then compare Incognito history and memory.</v>
+        <v>Select PDF, CSV, image, corrupted, empty, oversized, and password-protected fixtures; request analysis.</v>
       </c>
       <c r="G11" t="str">
-        <v>Normal memory persists; Incognito content does not persist or leak into memory.</v>
+        <v>Parsed content is accurate and invalid files return clear errors without silent failure.</v>
       </c>
       <c r="H11" t="str">
-        <v>Controls were verified, but a successful memory-setting conversation was unavailable for end-to-end verification.</v>
+        <v>Upload control accepted safe fixtures, but assistant-side parsing and full invalid-file processing were not completed.</v>
       </c>
       <c r="I11" t="str">
-        <v>tests/task01/memory-incognito.spec.ts; reports/task01/TASK-01-REPORT.md</v>
+        <v>tests/task01/upload-integrity.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
       <c r="J11" t="str">
-        <v>Memory panel opened; empty state observed; Incognito control visible and activatable.</v>
+        <v>Upload UI rendered PDF/CSV/SVG attachment chips; parsing request was not completed due to state-dependent limit.</v>
       </c>
       <c r="K11" t="str">
-        <v>Partial; state-dependent verification deferred</v>
+        <v>Partial; processing verification deferred</v>
       </c>
       <c r="L11" t="str">
-        <v>Repeat with a fresh usable conversation state; document server-backup deletion as client-side unverifiable.</v>
+        <v>Repeat with available message quota and controlled fixtures, then validate extracted values and errors.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>T01-F-004</v>
+        <v>T01-F-003</v>
       </c>
       <c r="B12" t="str">
         <v>Task 01</v>
@@ -846,75 +846,113 @@
         <v>Medium</v>
       </c>
       <c r="D12" t="str">
-        <v>Developer API funded behavior</v>
+        <v>Memory and Incognito</v>
       </c>
       <c r="E12" t="str">
-        <v>https://backend.thaura.ai/v1/chat/completions</v>
+        <v>https://thaura.ai/</v>
       </c>
       <c r="F12" t="str">
-        <v>Send minimal authenticated inference request with the dedicated API key.</v>
+        <v>Store a fact in normal mode, retrieve it in a new chat, then compare Incognito history and memory.</v>
       </c>
       <c r="G12" t="str">
-        <v>Funded key returns documented streaming/non-streaming response and usage schema.</v>
+        <v>Normal memory persists; Incognito content does not persist or leak into memory.</v>
       </c>
       <c r="H12" t="str">
-        <v>Key was recognized but returned documented 402 Insufficient balance; funded inference was unavailable.</v>
+        <v>Controls were verified, but a successful memory-setting conversation was unavailable for end-to-end verification.</v>
       </c>
       <c r="I12" t="str">
-        <v>tests/task01/developer-api-authenticated.spec.ts; reports/task01/TASK-01-REPORT.md</v>
+        <v>tests/task01/memory-incognito.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
       <c r="J12" t="str">
-        <v>POST /v1/chat/completions with accepted API key returned 402 Insufficient balance; invalid model returned 400.</v>
+        <v>Memory panel opened; empty state observed; Incognito control visible and activatable.</v>
       </c>
       <c r="K12" t="str">
-        <v>Partial; zero-balance verification boundary</v>
+        <v>Partial; state-dependent verification deferred</v>
       </c>
       <c r="L12" t="str">
-        <v>Repeat with an approved funded test key and minimal token budget.</v>
+        <v>Repeat with a fresh usable conversation state; document server-backup deletion as client-side unverifiable.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>T01-F-005</v>
+        <v>T01-F-004</v>
       </c>
       <c r="B13" t="str">
         <v>Task 01</v>
       </c>
       <c r="C13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Developer API funded behavior</v>
+      </c>
+      <c r="E13" t="str">
+        <v>https://backend.thaura.ai/v1/chat/completions</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Send minimal authenticated inference request with the dedicated API key.</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Funded key returns documented streaming/non-streaming response and usage schema.</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Key was recognized but returned documented 402 Insufficient balance; funded inference was unavailable.</v>
+      </c>
+      <c r="I13" t="str">
+        <v>tests/task01/developer-api-authenticated.spec.ts; reports/task01/TASK-01-REPORT.md</v>
+      </c>
+      <c r="J13" t="str">
+        <v>POST /v1/chat/completions with accepted API key returned 402 Insufficient balance; invalid model returned 400.</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Partial; zero-balance verification boundary</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Repeat with an approved funded test key and minimal token budget.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>T01-F-005</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Task 01</v>
+      </c>
+      <c r="C14" t="str">
         <v>Informational</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D14" t="str">
         <v>Settings/Account/Billing inputs</v>
       </c>
-      <c r="E13" t="str">
+      <c r="E14" t="str">
         <v>https://thaura.ai/</v>
       </c>
-      <c r="F13" t="str">
+      <c r="F14" t="str">
         <v>Open authenticated account controls and inspect Settings/Account/Billing forms.</v>
       </c>
-      <c r="G13" t="str">
+      <c r="G14" t="str">
         <v>Exposed fields are covered by negative and boundary tests.</v>
       </c>
-      <c r="H13" t="str">
+      <c r="H14" t="str">
         <v>No editable Settings/Account/Billing surface was exposed in the current UI probe.</v>
       </c>
-      <c r="I13" t="str">
+      <c r="I14" t="str">
         <v>tests/task01/negative-boundary.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
-      <c r="J13" t="str">
+      <c r="J14" t="str">
         <v>Authenticated UI probe exposed account menu but no editable Settings/Account/Billing form controls.</v>
       </c>
-      <c r="K13" t="str">
+      <c r="K14" t="str">
         <v>Deferred: surface not exposed</v>
       </c>
-      <c r="L13" t="str">
+      <c r="L14" t="str">
         <v>Locate the product routes or enable the relevant surface, then add field-level boundary tests.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L13"/>
+  <autoFilter ref="A1:L14"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -940,7 +978,7 @@
         <v>Total findings</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -956,7 +994,7 @@
         <v>Task 02 findings</v>
       </c>
       <c r="B4">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -964,7 +1002,7 @@
         <v>Confirmed defects/inconsistencies</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Refresh all Task 01/02 evidence; correct Firefox finding to intermittent
</commit_message>
<xml_diff>
--- a/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
+++ b/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
@@ -586,25 +586,25 @@
         <v>https://thaura.ai/</v>
       </c>
       <c r="F5" t="str">
-        <v>Run the compatibility project for Firefox desktop and wait for page hydration.</v>
+        <v>Run the compatibility project for Firefox desktop, repeated across multiple runs, and wait for page hydration.</v>
       </c>
       <c r="G5" t="str">
-        <v>Homepage renders usable content in Firefox.</v>
+        <v>Homepage reliably renders usable content in Firefox on every run.</v>
       </c>
       <c r="H5" t="str">
-        <v>Firefox returned 200 but remained on the loading spinner with no rendered body content.</v>
+        <v>Intermittent: 2026-09-17 retest showed 2 passes and 1 failure across 3 runs; on failure, Firefox returned 200 but remained on the loading spinner with no rendered body content.</v>
       </c>
       <c r="I5" t="str">
         <v>tests/task02/compatibility.spec.ts; reports/task02/TASK-02-BUG-REPORT.md</v>
       </c>
       <c r="J5" t="str">
-        <v>Firefox navigation returned HTTP 200; page remained on loading spinner and body content was empty.</v>
+        <v>Firefox navigation returned HTTP 200; intermittent on 2026-09-17 retest: 2 passes and 1 failure across 3 runs with empty body content on failure.</v>
       </c>
       <c r="K5" t="str">
-        <v>Confirmed compatibility failure</v>
+        <v>Confirmed intermittent compatibility issue</v>
       </c>
       <c r="L5" t="str">
-        <v>Investigate Firefox-specific hydration, JavaScript, or resource-loading behavior.</v>
+        <v>Investigate Firefox-specific hydration/timing race condition; not a hard incompatibility since it does not fail every run.</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Correct Task 01 quota finding and Task 02 Lighthouse/k6 figures from fresh evidence
</commit_message>
<xml_diff>
--- a/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
+++ b/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
@@ -776,25 +776,25 @@
         <v>https://thaura.ai/</v>
       </c>
       <c r="F10" t="str">
-        <v>Open a Free account after quota exhaustion and inspect the limit message.</v>
+        <v>Send 6 sequential prompts from a fresh Free-tier quota bucket and inspect the exact #5/#6 boundary and limit message.</v>
       </c>
       <c r="G10" t="str">
         <v>The documented 5-message/2-hour behavior is confirmed.</v>
       </c>
       <c r="H10" t="str">
-        <v>The product displayed 5 messages every 5 hours; a fresh #5/#6 boundary run was unavailable.</v>
+        <v>Messages 1-5 succeeded with responses; message 6 was blocked exactly at the boundary. The product displays 5 messages every 5 hours, not the assignment's stated 2-hour window.</v>
       </c>
       <c r="I10" t="str">
         <v>tests/task01/free-tier-quota.spec.ts; reports/task01/TASK-01-REPORT.md</v>
       </c>
       <c r="J10" t="str">
-        <v>Free account UI displayed: Out of messages; 5 messages every 5 hours; reset countdown approximately 5 hours.</v>
+        <v>Fresh quota-isolation run on 2026-09-17: Q1-Q5 returned 200 with responses; Q6 blocked with "5 messages every 5 hours"; reset countdown 4h 59m.</v>
       </c>
       <c r="K10" t="str">
-        <v>Partial; state-dependent verification deferred</v>
+        <v>Confirmed: exact boundary verified on a fresh quota bucket</v>
       </c>
       <c r="L10" t="str">
-        <v>Repeat with a genuinely fresh quota bucket and reconcile the product window with the assignment wording.</v>
+        <v>Reconcile the product's stated 5-hour reset window with the assignment's 2-hour wording.</v>
       </c>
     </row>
     <row r="11">
@@ -1002,7 +1002,7 @@
         <v>Confirmed defects/inconsistencies</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -1010,7 +1010,7 @@
         <v>Partial/deferred/blocked</v>
       </c>
       <c r="B6">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Lighthouse API-page audit to target public /api-platform route
</commit_message>
<xml_diff>
--- a/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
+++ b/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
@@ -697,28 +697,28 @@
         <v>Lighthouse API audit</v>
       </c>
       <c r="E8" t="str">
-        <v>https://thaura.ai/api</v>
+        <v>https://thaura.ai/api-platform; https://thaura.ai/api</v>
       </c>
       <c r="F8" t="str">
-        <v>Run the configured Lighthouse API audit anonymously.</v>
+        <v>Run the Lighthouse audit against the public API page (/api-platform) and, separately, against /api.</v>
       </c>
       <c r="G8" t="str">
-        <v>Key-page Lighthouse metrics are captured.</v>
+        <v>Key-page Lighthouse metrics are captured for the public-facing API page.</v>
       </c>
       <c r="H8" t="str">
-        <v>The route returned 401, so performance metrics were unavailable; /api-platform is the public documentation page.</v>
+        <v>/api-platform (the public, nav-linked API page) audited successfully with a 0.62 performance score. /api is a separate, non-public route that returns 401 regardless of authentication and is not the page referenced by the assignment.</v>
       </c>
       <c r="I8" t="str">
-        <v>reports/task02/lighthouse-api.json; README.md</v>
+        <v>reports/task02/lighthouse-api-platform.json; reports/task02/lighthouse-api.json</v>
       </c>
       <c r="J8" t="str">
-        <v>Lighthouse document request for /api returned 401 ERRORED_DOCUMENT_REQUEST.</v>
+        <v>/api-platform (the public API page) Lighthouse audit succeeded with performance score 0.62; /api (a protected, non-public route) returned 401 ERRORED_DOCUMENT_REQUEST.</v>
       </c>
       <c r="K8" t="str">
-        <v>Blocked by protected route</v>
+        <v>Resolved: correct public page identified and audited</v>
       </c>
       <c r="L8" t="str">
-        <v>Keep the 401 as evidence or audit /api-platform separately for public documentation performance.</v>
+        <v>Use /api-platform for API-page performance audits; treat /api's constant 401 as a separate access-control observation, not a performance-audit blocker.</v>
       </c>
     </row>
     <row r="9">
@@ -1010,7 +1010,7 @@
         <v>Partial/deferred/blocked</v>
       </c>
       <c r="B6">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Close Task 01 gaps: quota-bypass resistance test and PDF upload parsing-accuracy test
</commit_message>
<xml_diff>
--- a/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
+++ b/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Bug Register'!A1:L14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Bug Register'!A1:L16</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -949,10 +949,86 @@
         <v>Locate the product routes or enable the relevant surface, then add field-level boundary tests.</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>T01-F-006</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Task 01</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Informational</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Free-tier quota bypass resistance</v>
+      </c>
+      <c r="E15" t="str">
+        <v>https://thaura.ai/</v>
+      </c>
+      <c r="F15" t="str">
+        <v>On a fresh quota-exhausted account, attempt a second browser tab, a page refresh, and a direct replayed API call to POST /v1/chat/completions.</v>
+      </c>
+      <c r="G15" t="str">
+        <v>The account-wide quota block cannot be bypassed by any of the three vectors.</v>
+      </c>
+      <c r="H15" t="str">
+        <v>All three vectors remained blocked: second tab blocked, refreshed session still blocked, and the direct API replay returned 429 rate_limit_exceeded.</v>
+      </c>
+      <c r="I15" t="str">
+        <v>tests/task01/quota-bypass.spec.ts; reports/task01/TASK-01-REPORT.md</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Second-tab and refreshed-session attempts were both quota-blocked; a direct replayed API call returned 429 rate_limit_exceeded with a resetAt timestamp.</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Confirmed: quota cannot be bypassed via tested vectors</v>
+      </c>
+      <c r="L15" t="str">
+        <v>No action required; continue to enforce the limit server-side rather than relying on client state.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>T01-F-007</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Task 01</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Informational</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Upload parsing accuracy</v>
+      </c>
+      <c r="E16" t="str">
+        <v>https://thaura.ai/</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Attach known.pdf (containing the text "TASK01 PDF MARKER") and ask the assistant to reply with the exact marker text found inside it.</v>
+      </c>
+      <c r="G16" t="str">
+        <v>The assistant accurately extracts and reads back the document content, not just acknowledges the attachment.</v>
+      </c>
+      <c r="H16" t="str">
+        <v>The assistant replied with the exact marker text "TASK01 PDF MARKER", confirming accurate PDF content extraction.</v>
+      </c>
+      <c r="I16" t="str">
+        <v>tests/task01/upload-parsing-accuracy.spec.ts; reports/task01/TASK-01-REPORT.md</v>
+      </c>
+      <c r="J16" t="str">
+        <v>known.pdf (containing marker text "TASK01 PDF MARKER") was attached and the assistant replied with the exact marker text, confirming accurate content extraction.</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Confirmed: parsing accuracy verified for PDF text extraction</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Extend the same marker-based approach to spreadsheet and image fixtures for broader parsing-accuracy coverage.</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L14"/>
+  <autoFilter ref="A1:L16"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -978,7 +1054,7 @@
         <v>Total findings</v>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -986,7 +1062,7 @@
         <v>Task 01 findings</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -1002,7 +1078,7 @@
         <v>Confirmed defects/inconsistencies</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Add quota window-anchor and failed-response quota tests; fix live homepage-slowness impact on uploads
</commit_message>
<xml_diff>
--- a/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
+++ b/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Bug Register'!A1:L16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Bug Register'!A1:L19</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L19"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1025,10 +1025,124 @@
         <v>Extend the same marker-based approach to spreadsheet and image fixtures for broader parsing-accuracy coverage.</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>T01-F-008</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Task 01</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Informational</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Free-tier quota window behavior</v>
+      </c>
+      <c r="E17" t="str">
+        <v>https://thaura.ai/</v>
+      </c>
+      <c r="F17" t="str">
+        <v>On a fresh account, send 5 messages with recorded timestamps, then capture the resetAt timestamp from the 429 response on message 6.</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Determine whether the reset window is anchored to the oldest message (fixed) or extends with new activity (rolling).</v>
+      </c>
+      <c r="H17" t="str">
+        <v>resetAt was 21.5s from (first message + 5h) versus 25.6s from (last message + 5h); the window is anchored to the oldest message in the bucket, not extended by new activity.</v>
+      </c>
+      <c r="I17" t="str">
+        <v>tests/task01/quota-window-behavior.spec.ts; reports/task01/TASK-01-REPORT.md</v>
+      </c>
+      <c r="J17" t="str">
+        <v>resetAt=2026-09-17T20:32:52.923Z was 21.5s from (firstMessage+5h) vs 25.6s from (lastMessage+5h); the window is anchored to the oldest message.</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Confirmed: window is fixed/anchored to the oldest message</v>
+      </c>
+      <c r="L17" t="str">
+        <v>No action required; document this reset behavior for user-facing quota messaging.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>T01-F-009</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Task 01</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Informational</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Failed-request quota consumption</v>
+      </c>
+      <c r="E18" t="str">
+        <v>https://thaura.ai/</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Send a deliberately malformed completions request (messages as a string) on a fresh account, then send 5 legitimate messages via the UI.</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Determine whether a rejected/errored request still consumes one of the 5 allowed messages.</v>
+      </c>
+      <c r="H18" t="str">
+        <v>The malformed request returned 400; all 5 subsequent legitimate messages still succeeded without an early quota block.</v>
+      </c>
+      <c r="I18" t="str">
+        <v>tests/task01/quota-failed-response.spec.ts; reports/task01/TASK-01-REPORT.md</v>
+      </c>
+      <c r="J18" t="str">
+        <v>A malformed POST (messages as a string) returned 400 invalid_messages; all 5 subsequent legitimate messages still succeeded without an early quota block.</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Confirmed: errored requests do not consume a quota slot</v>
+      </c>
+      <c r="L18" t="str">
+        <v>No action required; only successfully-processed messages count against the Free-tier quota.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>T02-F-009</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Task 02</v>
+      </c>
+      <c r="C19" t="str">
+        <v>High</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Homepage performance/availability</v>
+      </c>
+      <c r="E19" t="str">
+        <v>https://thaura.ai/</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Navigate to the homepage in headless Chromium (anonymous and authenticated) and poll body content over time.</v>
+      </c>
+      <c r="G19" t="str">
+        <v>The homepage renders usable content within a few seconds, consistent with other public pages.</v>
+      </c>
+      <c r="H19" t="str">
+        <v>HTTP 200 returned but the body remained empty for 30-42+ seconds across repeated attempts on 2026-09-17; /faq and /pricing rendered normally within seconds in the same session. No console errors or failed requests were observed.</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Manual Playwright diagnostic script output, 2026-09-17; reports/task02/TASK-02-BUG-REPORT.md</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Homepage returned HTTP 200 with an empty rendered body for 30-42+ seconds across repeated attempts on 2026-09-17, while /faq and /pricing rendered normally within seconds.</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Confirmed live observation; may be transient, needs repeated sampling</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Investigate homepage-specific server-side rendering/data-fetch latency and add loading feedback or a timeout/fallback.</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L16"/>
+  <autoFilter ref="A1:L19"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1054,7 +1168,7 @@
         <v>Total findings</v>
       </c>
       <c r="B2">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -1062,7 +1176,7 @@
         <v>Task 01 findings</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -1070,7 +1184,7 @@
         <v>Task 02 findings</v>
       </c>
       <c r="B4">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -1078,7 +1192,7 @@
         <v>Confirmed defects/inconsistencies</v>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Correct F-006: attribute severe homepage-slowness measurement to local VPN, not a product defect
</commit_message>
<xml_diff>
--- a/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
+++ b/reports/TASK-01-TASK-02-BUG-REPORT.xlsx
@@ -1109,34 +1109,34 @@
         <v>Task 02</v>
       </c>
       <c r="C19" t="str">
-        <v>High</v>
+        <v>Low</v>
       </c>
       <c r="D19" t="str">
-        <v>Homepage performance/availability</v>
+        <v>Homepage performance</v>
       </c>
       <c r="E19" t="str">
         <v>https://thaura.ai/</v>
       </c>
       <c r="F19" t="str">
-        <v>Navigate to the homepage in headless Chromium (anonymous and authenticated) and poll body content over time.</v>
+        <v>Navigate to the homepage in headless Chromium (anonymous and authenticated) and poll body content over time; compare against /faq in the same session.</v>
       </c>
       <c r="G19" t="str">
-        <v>The homepage renders usable content within a few seconds, consistent with other public pages.</v>
+        <v>The homepage renders usable content within roughly the same time as other public pages.</v>
       </c>
       <c r="H19" t="str">
-        <v>HTTP 200 returned but the body remained empty for 30-42+ seconds across repeated attempts on 2026-09-17; /faq and /pricing rendered normally within seconds in the same session. No console errors or failed requests were observed.</v>
+        <v>Initial measurement: HTTP 200 with an empty body for 30-42+ seconds. After disabling a local VPN connection that had been active, a retest showed 5-17 seconds to render, versus ~4 seconds for /faq. No console errors or failed requests were observed in either measurement.</v>
       </c>
       <c r="I19" t="str">
-        <v>Manual Playwright diagnostic script output, 2026-09-17; reports/task02/TASK-02-BUG-REPORT.md</v>
+        <v>Manual Playwright diagnostic script output, 2026-09-17 (before and after VPN disabled); reports/task02/TASK-02-BUG-REPORT.md</v>
       </c>
       <c r="J19" t="str">
-        <v>Homepage returned HTTP 200 with an empty rendered body for 30-42+ seconds across repeated attempts on 2026-09-17, while /faq and /pricing rendered normally within seconds.</v>
+        <v>Initial measurement: homepage empty body for 30-42+ seconds. Retest after disabling local VPN: 5-17 seconds. Original severe result attributed to local network, not the product.</v>
       </c>
       <c r="K19" t="str">
-        <v>Confirmed live observation; may be transient, needs repeated sampling</v>
+        <v>Corrected: original severe result attributed to local VPN, not the product; small residual timing gap remains as a low-priority observation</v>
       </c>
       <c r="L19" t="str">
-        <v>Investigate homepage-specific server-side rendering/data-fetch latency and add loading feedback or a timeout/fallback.</v>
+        <v>Resample the residual homepage-vs-other-pages timing gap under confirmed clean network conditions before treating it as a product issue.</v>
       </c>
     </row>
   </sheetData>
@@ -1192,7 +1192,7 @@
         <v>Confirmed defects/inconsistencies</v>
       </c>
       <c r="B5">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">

</xml_diff>